<commit_message>
formatting and new item-names.csv
</commit_message>
<xml_diff>
--- a/references/Release9_DataDic/ESWAN.xlsx
+++ b/references/Release9_DataDic/ESWAN.xlsx
@@ -1,24 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="28410"/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/data/Research/Healthy Brain Network/Data Sharing/Data Dictionaries/Public Data Dictionaries/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Ksenia\Add Values\2files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="1880" yWindow="2120" windowWidth="25040" windowHeight="17820" tabRatio="500"/>
+    <workbookView xWindow="1884" yWindow="2124" windowWidth="25044" windowHeight="17820" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="140000" concurrentCalc="0"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
-      <x14:workbookPr defaultImageDpi="32767"/>
-    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -27,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="149">
   <si>
     <t>Question</t>
   </si>
@@ -508,7 +506,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -608,7 +606,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -616,7 +614,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -656,6 +653,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -984,29 +984,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F77"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="89.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="89.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="2" customFormat="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D1" s="3"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="4" t="s">
         <v>147</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
-      <c r="D2" s="6"/>
+      <c r="D2" s="5"/>
       <c r="E2" s="4"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
@@ -1016,33 +1016,33 @@
       <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="4" t="s">
         <v>129</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="6"/>
+      <c r="D4" s="5"/>
       <c r="E4" s="4"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:6">
+      <c r="A5" s="6" t="s">
         <v>130</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="7"/>
-    </row>
-    <row r="6" spans="1:6" ht="112" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+      <c r="D5" s="5"/>
+      <c r="E5" s="6"/>
+    </row>
+    <row r="6" spans="1:6" ht="109.2">
+      <c r="A6" s="6" t="s">
         <v>131</v>
       </c>
       <c r="B6" t="s">
@@ -1051,18 +1051,18 @@
       <c r="C6" t="s">
         <v>145</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="E6" s="15" t="s">
+      <c r="D6" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E6" s="14" t="s">
         <v>146</v>
       </c>
       <c r="F6" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+    <row r="7" spans="1:6" ht="109.2">
+      <c r="A7" s="6" t="s">
         <v>132</v>
       </c>
       <c r="B7" t="s">
@@ -1071,13 +1071,15 @@
       <c r="C7" t="s">
         <v>145</v>
       </c>
-      <c r="D7" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="13" t="s">
+      <c r="D7" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="109.2">
+      <c r="A8" s="12" t="s">
         <v>133</v>
       </c>
       <c r="B8" t="s">
@@ -1086,12 +1088,15 @@
       <c r="C8" t="s">
         <v>145</v>
       </c>
-      <c r="D8" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="13" t="s">
+      <c r="D8" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="109.2">
+      <c r="A9" s="12" t="s">
         <v>134</v>
       </c>
       <c r="B9" t="s">
@@ -1100,12 +1105,15 @@
       <c r="C9" t="s">
         <v>145</v>
       </c>
-      <c r="D9" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="12" t="s">
+      <c r="D9" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="109.2">
+      <c r="A10" s="11" t="s">
         <v>135</v>
       </c>
       <c r="B10" t="s">
@@ -1114,12 +1122,15 @@
       <c r="C10" t="s">
         <v>145</v>
       </c>
-      <c r="D10" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="13" t="s">
+      <c r="D10" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="109.2">
+      <c r="A11" s="12" t="s">
         <v>136</v>
       </c>
       <c r="B11" t="s">
@@ -1128,12 +1139,15 @@
       <c r="C11" t="s">
         <v>145</v>
       </c>
-      <c r="D11" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="13" t="s">
+      <c r="D11" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="109.2">
+      <c r="A12" s="12" t="s">
         <v>137</v>
       </c>
       <c r="B12" t="s">
@@ -1142,12 +1156,15 @@
       <c r="C12" t="s">
         <v>145</v>
       </c>
-      <c r="D12" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="13" t="s">
+      <c r="D12" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="109.2">
+      <c r="A13" s="12" t="s">
         <v>138</v>
       </c>
       <c r="B13" t="s">
@@ -1156,12 +1173,15 @@
       <c r="C13" t="s">
         <v>145</v>
       </c>
-      <c r="D13" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="13" t="s">
+      <c r="D13" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="109.2">
+      <c r="A14" s="12" t="s">
         <v>139</v>
       </c>
       <c r="B14" t="s">
@@ -1170,12 +1190,15 @@
       <c r="C14" t="s">
         <v>145</v>
       </c>
-      <c r="D14" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="13" t="s">
+      <c r="D14" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="109.2">
+      <c r="A15" s="12" t="s">
         <v>140</v>
       </c>
       <c r="B15" t="s">
@@ -1184,12 +1207,15 @@
       <c r="C15" t="s">
         <v>145</v>
       </c>
-      <c r="D15" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="13" t="s">
+      <c r="D15" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="109.2">
+      <c r="A16" s="12" t="s">
         <v>141</v>
       </c>
       <c r="B16" t="s">
@@ -1198,12 +1224,15 @@
       <c r="C16" t="s">
         <v>145</v>
       </c>
-      <c r="D16" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="13" t="s">
+      <c r="D16" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="109.2">
+      <c r="A17" s="12" t="s">
         <v>142</v>
       </c>
       <c r="B17" t="s">
@@ -1212,12 +1241,15 @@
       <c r="C17" t="s">
         <v>145</v>
       </c>
-      <c r="D17" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="13" t="s">
+      <c r="D17" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="109.2">
+      <c r="A18" s="12" t="s">
         <v>143</v>
       </c>
       <c r="B18" t="s">
@@ -1226,21 +1258,26 @@
       <c r="C18" t="s">
         <v>145</v>
       </c>
-      <c r="D18" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="10" t="s">
+      <c r="D18" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="9" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="12" t="s">
+      <c r="E19" s="14"/>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="11" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E20" s="14"/>
+    </row>
+    <row r="21" spans="1:5" ht="109.2">
       <c r="A21" t="s">
         <v>123</v>
       </c>
@@ -1250,11 +1287,14 @@
       <c r="C21" t="s">
         <v>145</v>
       </c>
-      <c r="D21" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D21" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="109.2">
       <c r="A22" t="s">
         <v>124</v>
       </c>
@@ -1264,11 +1304,14 @@
       <c r="C22" t="s">
         <v>145</v>
       </c>
-      <c r="D22" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D22" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="109.2">
       <c r="A23" t="s">
         <v>125</v>
       </c>
@@ -1278,11 +1321,14 @@
       <c r="C23" t="s">
         <v>145</v>
       </c>
-      <c r="D23" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D23" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="109.2">
       <c r="A24" t="s">
         <v>126</v>
       </c>
@@ -1292,11 +1338,14 @@
       <c r="C24" t="s">
         <v>145</v>
       </c>
-      <c r="D24" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D24" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="109.2">
       <c r="A25" t="s">
         <v>127</v>
       </c>
@@ -1306,11 +1355,14 @@
       <c r="C25" t="s">
         <v>145</v>
       </c>
-      <c r="D25" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D25" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="109.2">
       <c r="A26" t="s">
         <v>128</v>
       </c>
@@ -1320,29 +1372,36 @@
       <c r="C26" t="s">
         <v>145</v>
       </c>
-      <c r="D26" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D26" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="109.2">
       <c r="A27" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="4"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="7" t="s">
+      <c r="D27" s="5"/>
+      <c r="E27" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="109.2">
+      <c r="A28" s="6" t="s">
         <v>72</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="4"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D28" s="5"/>
+      <c r="E28" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="109.2">
       <c r="A29" t="s">
         <v>73</v>
       </c>
@@ -1352,11 +1411,14 @@
       <c r="C29" t="s">
         <v>145</v>
       </c>
-      <c r="D29" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D29" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="109.2">
       <c r="A30" t="s">
         <v>74</v>
       </c>
@@ -1366,11 +1428,14 @@
       <c r="C30" t="s">
         <v>145</v>
       </c>
-      <c r="D30" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D30" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="109.2">
       <c r="A31" t="s">
         <v>75</v>
       </c>
@@ -1380,11 +1445,14 @@
       <c r="C31" t="s">
         <v>145</v>
       </c>
-      <c r="D31" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D31" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="109.2">
       <c r="A32" t="s">
         <v>76</v>
       </c>
@@ -1394,11 +1462,14 @@
       <c r="C32" t="s">
         <v>145</v>
       </c>
-      <c r="D32" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D32" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="109.2">
       <c r="A33" t="s">
         <v>77</v>
       </c>
@@ -1408,11 +1479,14 @@
       <c r="C33" t="s">
         <v>145</v>
       </c>
-      <c r="D33" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D33" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="109.2">
       <c r="A34" t="s">
         <v>78</v>
       </c>
@@ -1422,11 +1496,14 @@
       <c r="C34" t="s">
         <v>145</v>
       </c>
-      <c r="D34" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D34" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="109.2">
       <c r="A35" t="s">
         <v>79</v>
       </c>
@@ -1436,11 +1513,14 @@
       <c r="C35" t="s">
         <v>145</v>
       </c>
-      <c r="D35" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D35" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="109.2">
       <c r="A36" t="s">
         <v>80</v>
       </c>
@@ -1450,11 +1530,14 @@
       <c r="C36" t="s">
         <v>145</v>
       </c>
-      <c r="D36" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D36" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="109.2">
       <c r="A37" t="s">
         <v>81</v>
       </c>
@@ -1464,11 +1547,14 @@
       <c r="C37" t="s">
         <v>145</v>
       </c>
-      <c r="D37" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D37" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="109.2">
       <c r="A38" t="s">
         <v>82</v>
       </c>
@@ -1478,11 +1564,14 @@
       <c r="C38" t="s">
         <v>145</v>
       </c>
-      <c r="D38" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D38" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="109.2">
       <c r="A39" t="s">
         <v>83</v>
       </c>
@@ -1492,11 +1581,14 @@
       <c r="C39" t="s">
         <v>145</v>
       </c>
-      <c r="D39" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D39" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E39" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="109.2">
       <c r="A40" t="s">
         <v>84</v>
       </c>
@@ -1506,11 +1598,14 @@
       <c r="C40" t="s">
         <v>145</v>
       </c>
-      <c r="D40" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D40" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E40" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="109.2">
       <c r="A41" t="s">
         <v>85</v>
       </c>
@@ -1520,11 +1615,14 @@
       <c r="C41" t="s">
         <v>145</v>
       </c>
-      <c r="D41" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D41" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="109.2">
       <c r="A42" t="s">
         <v>86</v>
       </c>
@@ -1534,11 +1632,14 @@
       <c r="C42" t="s">
         <v>145</v>
       </c>
-      <c r="D42" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D42" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E42" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="109.2">
       <c r="A43" t="s">
         <v>87</v>
       </c>
@@ -1548,11 +1649,14 @@
       <c r="C43" t="s">
         <v>145</v>
       </c>
-      <c r="D43" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D43" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E43" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="109.2">
       <c r="A44" t="s">
         <v>88</v>
       </c>
@@ -1562,11 +1666,14 @@
       <c r="C44" t="s">
         <v>145</v>
       </c>
-      <c r="D44" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D44" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E44" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="109.2">
       <c r="A45" t="s">
         <v>89</v>
       </c>
@@ -1576,11 +1683,14 @@
       <c r="C45" t="s">
         <v>145</v>
       </c>
-      <c r="D45" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D45" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E45" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="109.2">
       <c r="A46" t="s">
         <v>90</v>
       </c>
@@ -1590,11 +1700,14 @@
       <c r="C46" t="s">
         <v>145</v>
       </c>
-      <c r="D46" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D46" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="109.2">
       <c r="A47" t="s">
         <v>91</v>
       </c>
@@ -1604,11 +1717,14 @@
       <c r="C47" t="s">
         <v>145</v>
       </c>
-      <c r="D47" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D47" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E47" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="109.2">
       <c r="A48" t="s">
         <v>92</v>
       </c>
@@ -1618,11 +1734,14 @@
       <c r="C48" t="s">
         <v>145</v>
       </c>
-      <c r="D48" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D48" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="109.2">
       <c r="A49" t="s">
         <v>93</v>
       </c>
@@ -1632,11 +1751,14 @@
       <c r="C49" t="s">
         <v>145</v>
       </c>
-      <c r="D49" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D49" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E49" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="109.2">
       <c r="A50" t="s">
         <v>94</v>
       </c>
@@ -1646,11 +1768,14 @@
       <c r="C50" t="s">
         <v>145</v>
       </c>
-      <c r="D50" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D50" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E50" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="109.2">
       <c r="A51" t="s">
         <v>95</v>
       </c>
@@ -1660,11 +1785,14 @@
       <c r="C51" t="s">
         <v>145</v>
       </c>
-      <c r="D51" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D51" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="109.2">
       <c r="A52" t="s">
         <v>96</v>
       </c>
@@ -1674,11 +1802,14 @@
       <c r="C52" t="s">
         <v>145</v>
       </c>
-      <c r="D52" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D52" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="109.2">
       <c r="A53" t="s">
         <v>97</v>
       </c>
@@ -1688,11 +1819,14 @@
       <c r="C53" t="s">
         <v>145</v>
       </c>
-      <c r="D53" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D53" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E53" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="109.2">
       <c r="A54" t="s">
         <v>98</v>
       </c>
@@ -1702,11 +1836,14 @@
       <c r="C54" t="s">
         <v>145</v>
       </c>
-      <c r="D54" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D54" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E54" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="109.2">
       <c r="A55" t="s">
         <v>99</v>
       </c>
@@ -1716,12 +1853,15 @@
       <c r="C55" t="s">
         <v>145</v>
       </c>
-      <c r="D55" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A56" s="8" t="s">
+      <c r="D55" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E55" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="109.2">
+      <c r="A56" s="7" t="s">
         <v>100</v>
       </c>
       <c r="B56" t="s">
@@ -1730,12 +1870,15 @@
       <c r="C56" t="s">
         <v>145</v>
       </c>
-      <c r="D56" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A57" s="8" t="s">
+      <c r="D56" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E56" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="109.2">
+      <c r="A57" s="7" t="s">
         <v>101</v>
       </c>
       <c r="B57" t="s">
@@ -1744,12 +1887,15 @@
       <c r="C57" t="s">
         <v>145</v>
       </c>
-      <c r="D57" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A58" s="8" t="s">
+      <c r="D57" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E57" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="109.2">
+      <c r="A58" s="7" t="s">
         <v>102</v>
       </c>
       <c r="B58" t="s">
@@ -1758,22 +1904,27 @@
       <c r="C58" t="s">
         <v>145</v>
       </c>
-      <c r="D58" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="9" t="s">
+      <c r="D58" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E58" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" s="9" customFormat="1">
+      <c r="A59" s="8" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="11" t="s">
+      <c r="E59" s="14"/>
+    </row>
+    <row r="60" spans="1:5" s="9" customFormat="1">
+      <c r="A60" s="10" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="11" t="s">
+      <c r="E60" s="14"/>
+    </row>
+    <row r="61" spans="1:5" ht="109.2">
+      <c r="A61" s="10" t="s">
         <v>104</v>
       </c>
       <c r="B61" t="s">
@@ -1782,12 +1933,15 @@
       <c r="C61" t="s">
         <v>145</v>
       </c>
-      <c r="D61" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="11" t="s">
+      <c r="D61" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E61" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="109.2">
+      <c r="A62" s="10" t="s">
         <v>105</v>
       </c>
       <c r="B62" t="s">
@@ -1796,12 +1950,15 @@
       <c r="C62" t="s">
         <v>145</v>
       </c>
-      <c r="D62" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="11" t="s">
+      <c r="D62" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E62" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="109.2">
+      <c r="A63" s="10" t="s">
         <v>106</v>
       </c>
       <c r="B63" t="s">
@@ -1810,17 +1967,21 @@
       <c r="C63" t="s">
         <v>145</v>
       </c>
-      <c r="D63" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="32" x14ac:dyDescent="0.2">
-      <c r="A64" s="11" t="s">
+      <c r="D63" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E63" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="31.2">
+      <c r="A64" s="10" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="11" t="s">
+      <c r="E64" s="14"/>
+    </row>
+    <row r="65" spans="1:5" ht="109.2">
+      <c r="A65" s="10" t="s">
         <v>108</v>
       </c>
       <c r="B65" t="s">
@@ -1829,12 +1990,15 @@
       <c r="C65" t="s">
         <v>145</v>
       </c>
-      <c r="D65" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="11" t="s">
+      <c r="D65" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E65" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="109.2">
+      <c r="A66" s="10" t="s">
         <v>109</v>
       </c>
       <c r="B66" t="s">
@@ -1843,12 +2007,15 @@
       <c r="C66" t="s">
         <v>145</v>
       </c>
-      <c r="D66" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="11" t="s">
+      <c r="D66" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E66" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="109.2">
+      <c r="A67" s="10" t="s">
         <v>110</v>
       </c>
       <c r="B67" t="s">
@@ -1857,12 +2024,15 @@
       <c r="C67" t="s">
         <v>145</v>
       </c>
-      <c r="D67" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="11" t="s">
+      <c r="D67" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E67" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="109.2">
+      <c r="A68" s="10" t="s">
         <v>111</v>
       </c>
       <c r="B68" t="s">
@@ -1871,12 +2041,15 @@
       <c r="C68" t="s">
         <v>145</v>
       </c>
-      <c r="D68" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="11" t="s">
+      <c r="D68" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E68" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="109.2">
+      <c r="A69" s="10" t="s">
         <v>112</v>
       </c>
       <c r="B69" t="s">
@@ -1885,12 +2058,15 @@
       <c r="C69" t="s">
         <v>145</v>
       </c>
-      <c r="D69" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="11" t="s">
+      <c r="D69" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E69" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="109.2">
+      <c r="A70" s="10" t="s">
         <v>113</v>
       </c>
       <c r="B70" t="s">
@@ -1899,12 +2075,15 @@
       <c r="C70" t="s">
         <v>145</v>
       </c>
-      <c r="D70" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="11" t="s">
+      <c r="D70" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E70" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="109.2">
+      <c r="A71" s="10" t="s">
         <v>114</v>
       </c>
       <c r="B71" t="s">
@@ -1913,12 +2092,15 @@
       <c r="C71" t="s">
         <v>145</v>
       </c>
-      <c r="D71" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="11" t="s">
+      <c r="D71" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E71" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="109.2">
+      <c r="A72" s="10" t="s">
         <v>115</v>
       </c>
       <c r="B72" t="s">
@@ -1927,12 +2109,15 @@
       <c r="C72" t="s">
         <v>145</v>
       </c>
-      <c r="D72" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="11" t="s">
+      <c r="D72" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E72" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="109.2">
+      <c r="A73" s="10" t="s">
         <v>116</v>
       </c>
       <c r="B73" t="s">
@@ -1941,12 +2126,15 @@
       <c r="C73" t="s">
         <v>145</v>
       </c>
-      <c r="D73" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="11" t="s">
+      <c r="D73" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E73" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="109.2">
+      <c r="A74" s="10" t="s">
         <v>117</v>
       </c>
       <c r="B74" t="s">
@@ -1955,12 +2143,15 @@
       <c r="C74" t="s">
         <v>145</v>
       </c>
-      <c r="D74" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="11" t="s">
+      <c r="D74" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E74" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="109.2">
+      <c r="A75" s="10" t="s">
         <v>118</v>
       </c>
       <c r="B75" t="s">
@@ -1969,12 +2160,15 @@
       <c r="C75" t="s">
         <v>145</v>
       </c>
-      <c r="D75" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="11" t="s">
+      <c r="D75" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E75" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="109.2">
+      <c r="A76" s="10" t="s">
         <v>119</v>
       </c>
       <c r="B76" t="s">
@@ -1983,12 +2177,15 @@
       <c r="C76" t="s">
         <v>145</v>
       </c>
-      <c r="D76" s="14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="11" t="s">
+      <c r="D76" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E76" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" ht="109.2">
+      <c r="A77" s="10" t="s">
         <v>120</v>
       </c>
       <c r="B77" t="s">
@@ -1997,12 +2194,24 @@
       <c r="C77" t="s">
         <v>145</v>
       </c>
-      <c r="D77" s="14" t="s">
-        <v>144</v>
+      <c r="D77" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E77" s="14" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.6"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
new data dicts for inverse response options + rename make_HBN
</commit_message>
<xml_diff>
--- a/references/Release9_DataDic/ESWAN.xlsx
+++ b/references/Release9_DataDic/ESWAN.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10811"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Ksenia\Add Values\2files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/home/Repos/hbn/diagnosis_predictor/references/Release9_DataDic/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{826E0435-1392-144F-B1E0-7E7AC4BABCE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1884" yWindow="2124" windowWidth="25044" windowHeight="17820" tabRatio="500"/>
+    <workbookView xWindow="80" yWindow="580" windowWidth="18580" windowHeight="17340" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -487,26 +488,26 @@
     <t>Numeric</t>
   </si>
   <si>
+    <t>*In order to calculate the score for each assessment, calculate the average of the item values</t>
+  </si>
+  <si>
+    <t>*Applies to all questions</t>
+  </si>
+  <si>
     <t>-3= Far above average
 -2= Above average
 -1= Slightly above average
 0= Average
 1= Slightly below average
-2= Above average
-3= Far above average</t>
-  </si>
-  <si>
-    <t>*In order to calculate the score for each assessment, calculate the average of the item values</t>
-  </si>
-  <si>
-    <t>*Applies to all questions</t>
+2= Below average
+3= Far below average</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="7">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -606,32 +607,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -982,31 +976,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F77"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="89.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="89.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" ht="21">
+    <row r="1" spans="1:6" s="2" customFormat="1" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D1" s="3"/>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="5"/>
       <c r="E2" s="4"/>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
@@ -1023,7 +1017,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>129</v>
       </c>
@@ -1032,17 +1026,16 @@
       <c r="D4" s="5"/>
       <c r="E4" s="4"/>
     </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="6" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>130</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="5"/>
-      <c r="E5" s="6"/>
-    </row>
-    <row r="6" spans="1:6" ht="109.2">
-      <c r="A6" s="6" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>131</v>
       </c>
       <c r="B6" t="s">
@@ -1051,18 +1044,18 @@
       <c r="C6" t="s">
         <v>145</v>
       </c>
-      <c r="D6" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>146</v>
+      <c r="D6" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>148</v>
       </c>
       <c r="F6" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="109.2">
-      <c r="A7" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>132</v>
       </c>
       <c r="B7" t="s">
@@ -1071,15 +1064,15 @@
       <c r="C7" t="s">
         <v>145</v>
       </c>
-      <c r="D7" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="109.2">
-      <c r="A8" s="12" t="s">
+      <c r="D7" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>133</v>
       </c>
       <c r="B8" t="s">
@@ -1088,15 +1081,15 @@
       <c r="C8" t="s">
         <v>145</v>
       </c>
-      <c r="D8" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="109.2">
-      <c r="A9" s="12" t="s">
+      <c r="D8" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>134</v>
       </c>
       <c r="B9" t="s">
@@ -1105,15 +1098,15 @@
       <c r="C9" t="s">
         <v>145</v>
       </c>
-      <c r="D9" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="109.2">
-      <c r="A10" s="11" t="s">
+      <c r="D9" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>135</v>
       </c>
       <c r="B10" t="s">
@@ -1122,15 +1115,15 @@
       <c r="C10" t="s">
         <v>145</v>
       </c>
-      <c r="D10" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="109.2">
-      <c r="A11" s="12" t="s">
+      <c r="D10" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>136</v>
       </c>
       <c r="B11" t="s">
@@ -1139,15 +1132,15 @@
       <c r="C11" t="s">
         <v>145</v>
       </c>
-      <c r="D11" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="109.2">
-      <c r="A12" s="12" t="s">
+      <c r="D11" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>137</v>
       </c>
       <c r="B12" t="s">
@@ -1156,15 +1149,15 @@
       <c r="C12" t="s">
         <v>145</v>
       </c>
-      <c r="D12" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="109.2">
-      <c r="A13" s="12" t="s">
+      <c r="D12" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>138</v>
       </c>
       <c r="B13" t="s">
@@ -1173,15 +1166,15 @@
       <c r="C13" t="s">
         <v>145</v>
       </c>
-      <c r="D13" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="109.2">
-      <c r="A14" s="12" t="s">
+      <c r="D13" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>139</v>
       </c>
       <c r="B14" t="s">
@@ -1190,15 +1183,15 @@
       <c r="C14" t="s">
         <v>145</v>
       </c>
-      <c r="D14" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="109.2">
-      <c r="A15" s="12" t="s">
+      <c r="D14" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>140</v>
       </c>
       <c r="B15" t="s">
@@ -1207,15 +1200,15 @@
       <c r="C15" t="s">
         <v>145</v>
       </c>
-      <c r="D15" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="109.2">
-      <c r="A16" s="12" t="s">
+      <c r="D15" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>141</v>
       </c>
       <c r="B16" t="s">
@@ -1224,15 +1217,15 @@
       <c r="C16" t="s">
         <v>145</v>
       </c>
-      <c r="D16" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="109.2">
-      <c r="A17" s="12" t="s">
+      <c r="D16" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>142</v>
       </c>
       <c r="B17" t="s">
@@ -1241,15 +1234,15 @@
       <c r="C17" t="s">
         <v>145</v>
       </c>
-      <c r="D17" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="109.2">
-      <c r="A18" s="12" t="s">
+      <c r="D17" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>143</v>
       </c>
       <c r="B18" t="s">
@@ -1258,26 +1251,26 @@
       <c r="C18" t="s">
         <v>145</v>
       </c>
-      <c r="D18" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="9" t="s">
+      <c r="D18" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="E19" s="14"/>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="11" t="s">
+      <c r="E19" s="9"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>122</v>
       </c>
-      <c r="E20" s="14"/>
-    </row>
-    <row r="21" spans="1:5" ht="109.2">
+      <c r="E20" s="9"/>
+    </row>
+    <row r="21" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>123</v>
       </c>
@@ -1287,14 +1280,14 @@
       <c r="C21" t="s">
         <v>145</v>
       </c>
-      <c r="D21" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="109.2">
+      <c r="D21" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>124</v>
       </c>
@@ -1304,14 +1297,14 @@
       <c r="C22" t="s">
         <v>145</v>
       </c>
-      <c r="D22" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="109.2">
+      <c r="D22" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>125</v>
       </c>
@@ -1321,14 +1314,14 @@
       <c r="C23" t="s">
         <v>145</v>
       </c>
-      <c r="D23" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="109.2">
+      <c r="D23" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>126</v>
       </c>
@@ -1338,14 +1331,14 @@
       <c r="C24" t="s">
         <v>145</v>
       </c>
-      <c r="D24" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E24" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="109.2">
+      <c r="D24" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>127</v>
       </c>
@@ -1355,14 +1348,14 @@
       <c r="C25" t="s">
         <v>145</v>
       </c>
-      <c r="D25" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="109.2">
+      <c r="D25" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>128</v>
       </c>
@@ -1372,36 +1365,32 @@
       <c r="C26" t="s">
         <v>145</v>
       </c>
-      <c r="D26" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E26" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="109.2">
+      <c r="D26" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="5"/>
-      <c r="E27" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="109.2">
-      <c r="A28" s="6" t="s">
+      <c r="E27" s="9"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>72</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="5"/>
-      <c r="E28" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="109.2">
+      <c r="E28" s="9"/>
+    </row>
+    <row r="29" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>73</v>
       </c>
@@ -1411,14 +1400,14 @@
       <c r="C29" t="s">
         <v>145</v>
       </c>
-      <c r="D29" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E29" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="109.2">
+      <c r="D29" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>74</v>
       </c>
@@ -1428,14 +1417,14 @@
       <c r="C30" t="s">
         <v>145</v>
       </c>
-      <c r="D30" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E30" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="109.2">
+      <c r="D30" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>75</v>
       </c>
@@ -1445,14 +1434,14 @@
       <c r="C31" t="s">
         <v>145</v>
       </c>
-      <c r="D31" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E31" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="109.2">
+      <c r="D31" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>76</v>
       </c>
@@ -1462,14 +1451,14 @@
       <c r="C32" t="s">
         <v>145</v>
       </c>
-      <c r="D32" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E32" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="109.2">
+      <c r="D32" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>77</v>
       </c>
@@ -1479,14 +1468,14 @@
       <c r="C33" t="s">
         <v>145</v>
       </c>
-      <c r="D33" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E33" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="109.2">
+      <c r="D33" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>78</v>
       </c>
@@ -1496,14 +1485,14 @@
       <c r="C34" t="s">
         <v>145</v>
       </c>
-      <c r="D34" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E34" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="109.2">
+      <c r="D34" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>79</v>
       </c>
@@ -1513,14 +1502,14 @@
       <c r="C35" t="s">
         <v>145</v>
       </c>
-      <c r="D35" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E35" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="109.2">
+      <c r="D35" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>80</v>
       </c>
@@ -1530,14 +1519,14 @@
       <c r="C36" t="s">
         <v>145</v>
       </c>
-      <c r="D36" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E36" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="109.2">
+      <c r="D36" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>81</v>
       </c>
@@ -1547,14 +1536,14 @@
       <c r="C37" t="s">
         <v>145</v>
       </c>
-      <c r="D37" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E37" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="109.2">
+      <c r="D37" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>82</v>
       </c>
@@ -1564,14 +1553,14 @@
       <c r="C38" t="s">
         <v>145</v>
       </c>
-      <c r="D38" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="109.2">
+      <c r="D38" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>83</v>
       </c>
@@ -1581,14 +1570,14 @@
       <c r="C39" t="s">
         <v>145</v>
       </c>
-      <c r="D39" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E39" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="109.2">
+      <c r="D39" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>84</v>
       </c>
@@ -1598,14 +1587,14 @@
       <c r="C40" t="s">
         <v>145</v>
       </c>
-      <c r="D40" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E40" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="109.2">
+      <c r="D40" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>85</v>
       </c>
@@ -1615,14 +1604,14 @@
       <c r="C41" t="s">
         <v>145</v>
       </c>
-      <c r="D41" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="109.2">
+      <c r="D41" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>86</v>
       </c>
@@ -1632,14 +1621,14 @@
       <c r="C42" t="s">
         <v>145</v>
       </c>
-      <c r="D42" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E42" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="109.2">
+      <c r="D42" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>87</v>
       </c>
@@ -1649,14 +1638,14 @@
       <c r="C43" t="s">
         <v>145</v>
       </c>
-      <c r="D43" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E43" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="109.2">
+      <c r="D43" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>88</v>
       </c>
@@ -1666,14 +1655,14 @@
       <c r="C44" t="s">
         <v>145</v>
       </c>
-      <c r="D44" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E44" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="109.2">
+      <c r="D44" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>89</v>
       </c>
@@ -1683,14 +1672,14 @@
       <c r="C45" t="s">
         <v>145</v>
       </c>
-      <c r="D45" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E45" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="109.2">
+      <c r="D45" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>90</v>
       </c>
@@ -1700,14 +1689,14 @@
       <c r="C46" t="s">
         <v>145</v>
       </c>
-      <c r="D46" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E46" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="109.2">
+      <c r="D46" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>91</v>
       </c>
@@ -1717,14 +1706,14 @@
       <c r="C47" t="s">
         <v>145</v>
       </c>
-      <c r="D47" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E47" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="109.2">
+      <c r="D47" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>92</v>
       </c>
@@ -1734,14 +1723,14 @@
       <c r="C48" t="s">
         <v>145</v>
       </c>
-      <c r="D48" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E48" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="109.2">
+      <c r="D48" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>93</v>
       </c>
@@ -1751,14 +1740,14 @@
       <c r="C49" t="s">
         <v>145</v>
       </c>
-      <c r="D49" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E49" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="109.2">
+      <c r="D49" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>94</v>
       </c>
@@ -1768,14 +1757,14 @@
       <c r="C50" t="s">
         <v>145</v>
       </c>
-      <c r="D50" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E50" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" ht="109.2">
+      <c r="D50" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>95</v>
       </c>
@@ -1785,14 +1774,14 @@
       <c r="C51" t="s">
         <v>145</v>
       </c>
-      <c r="D51" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E51" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="109.2">
+      <c r="D51" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>96</v>
       </c>
@@ -1802,14 +1791,14 @@
       <c r="C52" t="s">
         <v>145</v>
       </c>
-      <c r="D52" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E52" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="109.2">
+      <c r="D52" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>97</v>
       </c>
@@ -1819,14 +1808,14 @@
       <c r="C53" t="s">
         <v>145</v>
       </c>
-      <c r="D53" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E53" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" ht="109.2">
+      <c r="D53" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>98</v>
       </c>
@@ -1836,14 +1825,14 @@
       <c r="C54" t="s">
         <v>145</v>
       </c>
-      <c r="D54" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E54" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="109.2">
+      <c r="D54" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E54" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="119" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>99</v>
       </c>
@@ -1853,15 +1842,15 @@
       <c r="C55" t="s">
         <v>145</v>
       </c>
-      <c r="D55" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E55" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="109.2">
-      <c r="A56" s="7" t="s">
+      <c r="D55" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A56" s="6" t="s">
         <v>100</v>
       </c>
       <c r="B56" t="s">
@@ -1870,15 +1859,15 @@
       <c r="C56" t="s">
         <v>145</v>
       </c>
-      <c r="D56" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E56" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" ht="109.2">
-      <c r="A57" s="7" t="s">
+      <c r="D56" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E56" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A57" s="6" t="s">
         <v>101</v>
       </c>
       <c r="B57" t="s">
@@ -1887,15 +1876,15 @@
       <c r="C57" t="s">
         <v>145</v>
       </c>
-      <c r="D57" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E57" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" ht="109.2">
-      <c r="A58" s="7" t="s">
+      <c r="D57" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A58" s="6" t="s">
         <v>102</v>
       </c>
       <c r="B58" t="s">
@@ -1904,27 +1893,31 @@
       <c r="C58" t="s">
         <v>145</v>
       </c>
-      <c r="D58" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E58" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" s="9" customFormat="1">
-      <c r="A59" s="8" t="s">
+      <c r="D58" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" s="4" customFormat="1" ht="119" x14ac:dyDescent="0.2">
+      <c r="A59" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E59" s="14"/>
-    </row>
-    <row r="60" spans="1:5" s="9" customFormat="1">
-      <c r="A60" s="10" t="s">
+      <c r="E59" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" s="4" customFormat="1" ht="119" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="E60" s="14"/>
-    </row>
-    <row r="61" spans="1:5" ht="109.2">
-      <c r="A61" s="10" t="s">
+      <c r="E60" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A61" s="6" t="s">
         <v>104</v>
       </c>
       <c r="B61" t="s">
@@ -1933,15 +1926,15 @@
       <c r="C61" t="s">
         <v>145</v>
       </c>
-      <c r="D61" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E61" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" ht="109.2">
-      <c r="A62" s="10" t="s">
+      <c r="D61" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A62" s="6" t="s">
         <v>105</v>
       </c>
       <c r="B62" t="s">
@@ -1950,15 +1943,15 @@
       <c r="C62" t="s">
         <v>145</v>
       </c>
-      <c r="D62" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E62" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" ht="109.2">
-      <c r="A63" s="10" t="s">
+      <c r="D62" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E62" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A63" s="6" t="s">
         <v>106</v>
       </c>
       <c r="B63" t="s">
@@ -1967,21 +1960,21 @@
       <c r="C63" t="s">
         <v>145</v>
       </c>
-      <c r="D63" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E63" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" ht="31.2">
-      <c r="A64" s="10" t="s">
+      <c r="D63" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E63" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A64" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="E64" s="14"/>
-    </row>
-    <row r="65" spans="1:5" ht="109.2">
-      <c r="A65" s="10" t="s">
+      <c r="E64" s="9"/>
+    </row>
+    <row r="65" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A65" s="6" t="s">
         <v>108</v>
       </c>
       <c r="B65" t="s">
@@ -1990,15 +1983,15 @@
       <c r="C65" t="s">
         <v>145</v>
       </c>
-      <c r="D65" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E65" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="109.2">
-      <c r="A66" s="10" t="s">
+      <c r="D65" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E65" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A66" s="6" t="s">
         <v>109</v>
       </c>
       <c r="B66" t="s">
@@ -2007,15 +2000,15 @@
       <c r="C66" t="s">
         <v>145</v>
       </c>
-      <c r="D66" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E66" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" ht="109.2">
-      <c r="A67" s="10" t="s">
+      <c r="D66" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E66" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A67" s="6" t="s">
         <v>110</v>
       </c>
       <c r="B67" t="s">
@@ -2024,15 +2017,15 @@
       <c r="C67" t="s">
         <v>145</v>
       </c>
-      <c r="D67" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E67" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="109.2">
-      <c r="A68" s="10" t="s">
+      <c r="D67" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E67" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A68" s="6" t="s">
         <v>111</v>
       </c>
       <c r="B68" t="s">
@@ -2041,15 +2034,15 @@
       <c r="C68" t="s">
         <v>145</v>
       </c>
-      <c r="D68" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E68" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" ht="109.2">
-      <c r="A69" s="10" t="s">
+      <c r="D68" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E68" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A69" s="6" t="s">
         <v>112</v>
       </c>
       <c r="B69" t="s">
@@ -2058,15 +2051,15 @@
       <c r="C69" t="s">
         <v>145</v>
       </c>
-      <c r="D69" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E69" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" ht="109.2">
-      <c r="A70" s="10" t="s">
+      <c r="D69" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E69" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A70" s="6" t="s">
         <v>113</v>
       </c>
       <c r="B70" t="s">
@@ -2075,15 +2068,15 @@
       <c r="C70" t="s">
         <v>145</v>
       </c>
-      <c r="D70" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E70" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" ht="109.2">
-      <c r="A71" s="10" t="s">
+      <c r="D70" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E70" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A71" s="6" t="s">
         <v>114</v>
       </c>
       <c r="B71" t="s">
@@ -2092,15 +2085,15 @@
       <c r="C71" t="s">
         <v>145</v>
       </c>
-      <c r="D71" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E71" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" ht="109.2">
-      <c r="A72" s="10" t="s">
+      <c r="D71" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E71" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A72" s="6" t="s">
         <v>115</v>
       </c>
       <c r="B72" t="s">
@@ -2109,15 +2102,15 @@
       <c r="C72" t="s">
         <v>145</v>
       </c>
-      <c r="D72" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E72" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" ht="109.2">
-      <c r="A73" s="10" t="s">
+      <c r="D72" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E72" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A73" s="6" t="s">
         <v>116</v>
       </c>
       <c r="B73" t="s">
@@ -2126,15 +2119,15 @@
       <c r="C73" t="s">
         <v>145</v>
       </c>
-      <c r="D73" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E73" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" ht="109.2">
-      <c r="A74" s="10" t="s">
+      <c r="D73" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E73" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A74" s="6" t="s">
         <v>117</v>
       </c>
       <c r="B74" t="s">
@@ -2143,15 +2136,15 @@
       <c r="C74" t="s">
         <v>145</v>
       </c>
-      <c r="D74" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E74" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" ht="109.2">
-      <c r="A75" s="10" t="s">
+      <c r="D74" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E74" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A75" s="6" t="s">
         <v>118</v>
       </c>
       <c r="B75" t="s">
@@ -2160,15 +2153,15 @@
       <c r="C75" t="s">
         <v>145</v>
       </c>
-      <c r="D75" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E75" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" ht="109.2">
-      <c r="A76" s="10" t="s">
+      <c r="D75" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E75" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A76" s="6" t="s">
         <v>119</v>
       </c>
       <c r="B76" t="s">
@@ -2177,15 +2170,15 @@
       <c r="C76" t="s">
         <v>145</v>
       </c>
-      <c r="D76" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E76" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" ht="109.2">
-      <c r="A77" s="10" t="s">
+      <c r="D76" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E76" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" ht="119" x14ac:dyDescent="0.2">
+      <c r="A77" s="6" t="s">
         <v>120</v>
       </c>
       <c r="B77" t="s">
@@ -2194,11 +2187,11 @@
       <c r="C77" t="s">
         <v>145</v>
       </c>
-      <c r="D77" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E77" s="14" t="s">
-        <v>146</v>
+      <c r="D77" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2208,9 +2201,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>